<commit_message>
Add analysis script and report; update dataset
Add BEFD_FinalProject_ZEYNEP_TUTAR.R containing the full OTT/cinema time series analysis: data import and imputation, EDA (plots, correlation, VIF), multiple models and forecasts (TSLM, stepwise, ARIMA/autoARIMA, SARIMAX, Bass, GBM, GBM+SARIMAX, Prophet, Prophet+ARIMA, Holt-Winters), performance metrics, and forecasting pipeline. Add BEFD_Project_Report_ZEYNEP_TUTAR.pdf (final project report). Update ott_cinema_dataset.xlsx (data changes).
</commit_message>
<xml_diff>
--- a/ott_cinema_dataset.xlsx
+++ b/ott_cinema_dataset.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d9d1c894097c761c/Masaüstü/UNIPD/2-1/BUSINESS^J ECONOMIC AND FINANCIAL DATA/BEFD_Final_Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d9d1c894097c761c/Masaüstü/UNIPD/2-2/BUSINESS^J ECONOMIC AND FINANCIAL DATA/BEFD_Final_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="72" documentId="8_{10E86178-9A90-4768-AB0F-543806C97FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{329F12DF-F898-4250-A2A1-59C3EB265EAA}"/>
@@ -1112,10 +1112,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>